<commit_message>
Taco Shop Checklists EN, revisión final: 11 xlsx remontados y volcados (VPS)
extraer_textos (c0053 pasa a GM, ids estables), heredar (457 pendientes), aplicar_en --idempotencia --mes October
(0 diferencias); gates VERDE 8/0, autotest 16/16, censo-entregables y no-latinos 0, LIT255 verde.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/taco-shop-checklist-templates/01-taco-shop-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/taco-shop-checklist-templates/01-taco-shop-opening-closing-checklists.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Light the trompo (vertical broiler) and check for an even flame on every burner. Gas smell: light nothing, flip no switches, get out and call the gas company or 911 from outside</t>
+          <t>Check the cone as received: frozen at 0 °F or below, or refrigerated at 41 °F or below</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>10:50 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="F13" s="13" t="n"/>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Check the cone as received: frozen at 0 °F or below, or refrigerated at 41 °F or below</t>
+          <t>Stack the day's trompo: layer order, fat, pineapple and onion; note weight and time</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>9:45 AM</t>
         </is>
       </c>
       <c r="F14" s="13" t="n"/>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Stack the day's trompo: layer order, fat, pineapple and onion; note weight and time</t>
+          <t>Light the trompo (vertical broiler) and check for an even flame on every burner. Gas smell: light nothing, flip no switches, get out and call the gas company or 911 from outside</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>11:05 AM</t>
+          <t>9:50 AM</t>
         </is>
       </c>
       <c r="F15" s="13" t="n"/>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Review the shift's reservations and large-party forecast</t>
+          <t>Review the shift's catering and large-order forecast</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Pull the leftover meat off the trompo and log where it went: cooled or tossed. Reuse only if your health department allows it (the county sets the leftover-cone rule). If kept: cool from 135 °F to 70 °F within 2 h and to 41 °F within 4 more hours, covered and date-marked, 7 days max at 41 °F (day 1 = prep day)</t>
+          <t>Pull the leftover meat off the trompo and log where it went: cooled or tossed. Reuse only if your health department allows it (the county sets the leftover-cone rule). If kept: cool from 135 °F to 70 °F within 2 h and to 41 °F within 4 more hours, covered and date-marked, 7 days max at 41 °F (day 1 = prep day); reheat to 165 °F within 2 h before it goes back to hot holding</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">

</xml_diff>